<commit_message>
IDMA exam registration and more
</commit_message>
<xml_diff>
--- a/ExamWritten_260408/ExamRegistration_IDMA26_NDAB23002E.xlsx
+++ b/ExamWritten_260408/ExamRegistration_IDMA26_NDAB23002E.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\SUN-FAK-Studienaevn-Eksamen\SCIENCE Nørre\5. Tilmeldingslister\2025-2026\Tilmeldingslister B3 ordinær\DIKU B3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\Teaching\IDMA26\ExamWritten_260408\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26018752-E129-4CA0-86CD-710595BA90DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9338CA37-014D-402C-ADED-06AE7D6A86F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{57A13A8E-65B9-4FA0-863F-C04F21F1EE5C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{57A13A8E-65B9-4FA0-863F-C04F21F1EE5C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1613" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1644" uniqueCount="377">
   <si>
     <t>ADM</t>
   </si>
@@ -1158,6 +1158,15 @@
   </si>
   <si>
     <t>MF (Skriv MF hvis MF, ellers blank)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    MF</t>
+  </si>
+  <si>
+    <t>Cannot find this student --- have sent e-mail</t>
+  </si>
+  <si>
+    <t>Cannot find this student, and e-mail bounces</t>
   </si>
 </sst>
 </file>
@@ -1641,7 +1650,9 @@
       <c r="I2" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="1"/>
+      <c r="K2" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -1791,7 +1802,9 @@
       <c r="I7" t="s">
         <v>17</v>
       </c>
-      <c r="K7" s="1"/>
+      <c r="K7" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -1971,7 +1984,9 @@
       <c r="I13" t="s">
         <v>17</v>
       </c>
-      <c r="K13" s="1"/>
+      <c r="K13" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -2361,7 +2376,9 @@
       <c r="I26" t="s">
         <v>17</v>
       </c>
-      <c r="K26" s="1"/>
+      <c r="K26" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
@@ -2661,7 +2678,9 @@
       <c r="I36" t="s">
         <v>17</v>
       </c>
-      <c r="K36" s="1"/>
+      <c r="K36" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
@@ -2781,7 +2800,9 @@
       <c r="I40" t="s">
         <v>17</v>
       </c>
-      <c r="K40" s="1"/>
+      <c r="K40" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
@@ -2901,7 +2922,9 @@
       <c r="I44" t="s">
         <v>17</v>
       </c>
-      <c r="K44" s="1"/>
+      <c r="K44" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
@@ -2961,7 +2984,9 @@
       <c r="I46" t="s">
         <v>17</v>
       </c>
-      <c r="K46" s="1"/>
+      <c r="K46" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
@@ -3111,7 +3136,9 @@
       <c r="I51" t="s">
         <v>17</v>
       </c>
-      <c r="K51" s="1"/>
+      <c r="K51" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
@@ -3261,7 +3288,9 @@
       <c r="I56" t="s">
         <v>17</v>
       </c>
-      <c r="K56" s="1"/>
+      <c r="K56" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
@@ -3621,7 +3650,9 @@
       <c r="I68" t="s">
         <v>17</v>
       </c>
-      <c r="K68" s="1"/>
+      <c r="K68" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
@@ -3651,7 +3682,9 @@
       <c r="I69" t="s">
         <v>17</v>
       </c>
-      <c r="K69" s="1"/>
+      <c r="K69" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
@@ -3681,7 +3714,9 @@
       <c r="I70" t="s">
         <v>17</v>
       </c>
-      <c r="K70" s="1"/>
+      <c r="K70" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
@@ -3741,7 +3776,9 @@
       <c r="I72" t="s">
         <v>17</v>
       </c>
-      <c r="K72" s="1"/>
+      <c r="K72" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
@@ -4041,7 +4078,9 @@
       <c r="I82" t="s">
         <v>17</v>
       </c>
-      <c r="K82" s="1"/>
+      <c r="K82" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
@@ -4071,7 +4110,9 @@
       <c r="I83" t="s">
         <v>17</v>
       </c>
-      <c r="K83" s="1"/>
+      <c r="K83" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
@@ -4221,7 +4262,9 @@
       <c r="I88" t="s">
         <v>17</v>
       </c>
-      <c r="K88" s="1"/>
+      <c r="K88" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
@@ -4521,7 +4564,9 @@
       <c r="I98" t="s">
         <v>17</v>
       </c>
-      <c r="K98" s="1"/>
+      <c r="K98" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
@@ -4851,7 +4896,9 @@
       <c r="I109" t="s">
         <v>17</v>
       </c>
-      <c r="K109" s="1"/>
+      <c r="K109" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
@@ -5211,7 +5258,9 @@
       <c r="I121" t="s">
         <v>17</v>
       </c>
-      <c r="K121" s="1"/>
+      <c r="K121" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
@@ -5421,7 +5470,9 @@
       <c r="I128" t="s">
         <v>17</v>
       </c>
-      <c r="K128" s="1"/>
+      <c r="K128" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="129" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
@@ -5451,7 +5502,9 @@
       <c r="I129" t="s">
         <v>17</v>
       </c>
-      <c r="K129" s="1"/>
+      <c r="K129" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="130" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
@@ -5571,7 +5624,9 @@
       <c r="I133" t="s">
         <v>17</v>
       </c>
-      <c r="K133" s="1"/>
+      <c r="K133" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="134" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
@@ -5841,7 +5896,9 @@
       <c r="I142" t="s">
         <v>17</v>
       </c>
-      <c r="K142" s="1"/>
+      <c r="K142" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="143" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
@@ -6051,7 +6108,9 @@
       <c r="I149" t="s">
         <v>17</v>
       </c>
-      <c r="K149" s="1"/>
+      <c r="K149" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="150" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
@@ -6171,7 +6230,9 @@
       <c r="I153" t="s">
         <v>17</v>
       </c>
-      <c r="K153" s="1"/>
+      <c r="K153" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="154" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
@@ -6201,7 +6262,9 @@
       <c r="I154" t="s">
         <v>17</v>
       </c>
-      <c r="K154" s="1"/>
+      <c r="K154" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="155" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
@@ -6261,7 +6324,9 @@
       <c r="I156" t="s">
         <v>17</v>
       </c>
-      <c r="K156" s="1"/>
+      <c r="K156" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="157" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
@@ -6861,7 +6926,9 @@
       <c r="I176" t="s">
         <v>17</v>
       </c>
-      <c r="K176" s="1"/>
+      <c r="K176" s="1" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="177" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
@@ -6891,7 +6958,9 @@
       <c r="I177" t="s">
         <v>17</v>
       </c>
-      <c r="K177" s="1"/>
+      <c r="K177" s="1" t="s">
+        <v>376</v>
+      </c>
     </row>
     <row r="178" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
@@ -6921,7 +6990,9 @@
       <c r="I178" t="s">
         <v>17</v>
       </c>
-      <c r="K178" s="1"/>
+      <c r="K178" s="1" t="s">
+        <v>375</v>
+      </c>
     </row>
     <row r="179" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A179" t="s">

</xml_diff>